<commit_message>
feat(export): reconcile handover template export API with updated placeholders sheet
- Updated export API route to match new Placeholders sheet structure
- Mapped 19 placeholder rows to database fields (counteragent, insider, project)
- Skipped rows 5, 16, 18 to preserve formulas (genitive conversion, contract date)
- Template now has 19 rows with proper column A names and empty Column B values
- Verified TypeScript compilation and ESLint checks pass

[skip ci]
</commit_message>
<xml_diff>
--- a/public/handover template.xlsx
+++ b/public/handover template.xlsx
@@ -5,19 +5,42 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\next-postgres-starter\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\next-postgres-starter\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76EC226C-4514-4FDC-B70C-4753488A42C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23B65B36-C0E6-432A-81F3-F0556A51AAA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Handover" sheetId="4" r:id="rId1"/>
-    <sheet name="Jobs" sheetId="1" r:id="rId2"/>
-    <sheet name="Income Payments" sheetId="2" r:id="rId3"/>
-    <sheet name="Job Distributions" sheetId="3" r:id="rId4"/>
+    <sheet name="Placeholders" sheetId="5" r:id="rId2"/>
+    <sheet name="Jobs" sheetId="1" r:id="rId3"/>
+    <sheet name="Income Payments" sheetId="2" r:id="rId4"/>
+    <sheet name="Job Distributions" sheetId="3" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName name="Contract_Date">Placeholders!$B$18</definedName>
+    <definedName name="Handover_Date">Placeholders!$B$2</definedName>
+    <definedName name="Nominal_Handover_Price">Handover!$J$17:$J$64</definedName>
+    <definedName name="Project_Address">Placeholders!$B$10</definedName>
+    <definedName name="Project_Counteragent_Address_Line_1">Placeholders!$B$7</definedName>
+    <definedName name="Project_Counteragent_Address_Line_2">Placeholders!$B$8</definedName>
+    <definedName name="Project_Counteragent_Director">Placeholders!$B$6</definedName>
+    <definedName name="Project_Counteragent_Director_Genitive">Placeholders!$B$5</definedName>
+    <definedName name="Project_Counteragent_Entity_Type">Placeholders!$B$3</definedName>
+    <definedName name="Project_Counteragent_ID">Placeholders!$B$9</definedName>
+    <definedName name="Project_Counteragent_Name">Placeholders!$B$4</definedName>
+    <definedName name="Project_Currency">Placeholders!$B$19</definedName>
+    <definedName name="Project_Department">Placeholders!$B$1</definedName>
+    <definedName name="Project_Insider_Address_Line1">Placeholders!$B$14</definedName>
+    <definedName name="Project_Insider_Address_Line2">Placeholders!$B$15</definedName>
+    <definedName name="Project_Insider_Director_Genitive">Placeholders!$B$16</definedName>
+    <definedName name="Project_Insider_Director_Normative">Placeholders!$B$17</definedName>
+    <definedName name="Project_Insider_Entity_Type">Placeholders!$B$11</definedName>
+    <definedName name="Project_Insider_ID">Placeholders!$B$13</definedName>
+    <definedName name="Project_Insider_Name">Placeholders!$B$12</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -38,8 +61,9 @@
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
 <metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
+  <metadataTypes count="2">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
   <futureMetadata name="XLDAPR" count="1">
     <bk>
@@ -50,16 +74,40 @@
       </extLst>
     </bk>
   </futureMetadata>
+  <futureMetadata name="XLRICHVALUE" count="2">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="1"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
   <cellMetadata count="1">
     <bk>
       <rc t="1" v="0"/>
     </bk>
   </cellMetadata>
+  <valueMetadata count="2">
+    <bk>
+      <rc t="2" v="0"/>
+    </bk>
+    <bk>
+      <rc t="2" v="1"/>
+    </bk>
+  </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="105">
   <si>
     <t>Job Name</t>
   </si>
@@ -289,27 +337,13 @@
     <t>მიღება-ჩაბარების აქტი</t>
   </si>
   <si>
-    <t>Comment: if project department = Batumi, then "ქ. ბათუმი", if project department = Batumi, then "ქ. თბილისი"</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 	"ერთი მხრივ" + project.counteragent.entity_type.Name_Geo +  project.counteragent.Name +" -  წარმოდგენილი დირექტორის" + project.counteragent.Director_name+" (შემდგომში „დამკვეთი“)". მისამართი: "+  project.counteragent.address + " საიდენტიფიკაციო ნომერი: " + project.counteragent.id.
-             "მეორე მხრივ, შპს „აი-სი-ი“ წარმოდგენილი დირექტორის  გიორგი ბახტაძის სახით (შემდგომში „კონტრაქტორი“). მისამართი: ქ. თბილისი,ვაკის რაიონი, ზურაბ ანჯაფარიძის I შესახვევი N 4, საიდენტიფიკაციო ნომერი:  400017245."
-              "ვადგენთ წინამდებარე აქტს მასზედ, რომ შემსრულებელმა მიაწოდა, ხოლო დამკვეთმა მიიღო," +  if (project department = Batumi, then "ქ. ბათუმში", if project department = Tbuilisi, then "ქ. თბილიში," + Project.address + "-ში    „დამკვეთის“ სამშენებლო ტერიტორიაზე შემდეგი ლიფტები:</t>
-  </si>
-  <si>
     <t>#</t>
   </si>
   <si>
     <t>მწარმოებელი</t>
   </si>
   <si>
-    <t>თანხა + symbol lookup for the nominal  currency, if it is USD than $, is</t>
-  </si>
-  <si>
     <t>თანხა ₾</t>
-  </si>
-  <si>
-    <t>Comment : Certificate Date in format dd თვე სრულად ქართულად yyyy წელი (the handover should depict only one date at once, so if there are multiple dates in certificates users should celect a date and only that day's certified jobs should persist in the handover act) for this example I will use 27.05.2026</t>
   </si>
   <si>
     <t>ჯამი</t>
@@ -338,24 +372,61 @@
 3. წინამდებარე აქტი შედგენილია თანაბარი იურიდიული ძალის მქონე 2 (ორი) ეგზემპლარად, ერთი ეგზემპლარი გადაეცემა დამკვეთს, ხოლო ერთი - შემსრულებელს.</t>
   </si>
   <si>
-    <t xml:space="preserve"> 
-project.counteragent.entity_type.Name_Geo +  project.counteragent.Name 
-(დამკვეთი)
-----------------------------------
-დირექტორი 
-project.counteragent.Director_name
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  
-            შპს აი-სი-ი
-        (შემსრულებელი)
-           --------------------------------
-           დირექტორი
-           გიორგი ბახტაძე</t>
-  </si>
-  <si>
-    <t>თარიღი:</t>
+    <t>Project_Department</t>
+  </si>
+  <si>
+    <t>Handover_Date</t>
+  </si>
+  <si>
+    <t>Project_Counteragent_Entity_Type</t>
+  </si>
+  <si>
+    <t>Project_Counteragent_Name</t>
+  </si>
+  <si>
+    <t>Project_Counteragent_Address_Line_1</t>
+  </si>
+  <si>
+    <t>Project_Counteragent_Address_Line_2</t>
+  </si>
+  <si>
+    <t>Project_Counteragent_Director</t>
+  </si>
+  <si>
+    <t>Project_Counteragent_ID</t>
+  </si>
+  <si>
+    <t>Project_Address</t>
+  </si>
+  <si>
+    <t>Project_Counteragent_Director_Genitive</t>
+  </si>
+  <si>
+    <t>Project_Insider_Entity_Type</t>
+  </si>
+  <si>
+    <t>Project_Insider_Name</t>
+  </si>
+  <si>
+    <t>Project_Insider_Address_Line1</t>
+  </si>
+  <si>
+    <t>Project_Insider_Address_Line2</t>
+  </si>
+  <si>
+    <t>Project_Insider_Director_Genitive</t>
+  </si>
+  <si>
+    <t>Project_Insider_Director_Normative</t>
+  </si>
+  <si>
+    <t>Contract_Date</t>
+  </si>
+  <si>
+    <t>Project_Currency</t>
+  </si>
+  <si>
+    <t>Project_Insider_ID</t>
   </si>
 </sst>
 </file>
@@ -364,10 +435,10 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="dd\.mm\.yyyy"/>
-    <numFmt numFmtId="171" formatCode="dd\.mm\.yyyy;@"/>
+    <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
+    <numFmt numFmtId="165" formatCode="dd\.mm\.yyyy;@"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -396,8 +467,14 @@
       <name val="Sylfaen"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -407,6 +484,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -439,27 +522,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="justify" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -469,9 +540,6 @@
     <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -479,11 +547,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="justify" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="justify"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -491,8 +560,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="justify"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -510,6 +597,76 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
+  <rv s="0">
+    <v>8</v>
+    <v>1</v>
+  </rv>
+  <rv s="1">
+    <v>0</v>
+    <v>8</v>
+    <v>1</v>
+    <v>3</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
+  <s t="_error">
+    <k n="errorType" t="i"/>
+    <k n="propagated" t="b"/>
+  </s>
+  <s t="_error">
+    <k n="colOffset" t="i"/>
+    <k n="errorType" t="i"/>
+    <k n="rwOffset" t="i"/>
+    <k n="subType" t="i"/>
+  </s>
+</rvStructures>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -834,7 +991,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC07BC11-7207-41CD-A3C8-355D7D7D75EF}">
-  <dimension ref="C1:AC85"/>
+  <sheetPr codeName="Sheet1"/>
+  <dimension ref="C1:W85"/>
   <sheetFormatPr defaultColWidth="2.625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="4.5" customWidth="1"/>
@@ -846,901 +1004,889 @@
     <col min="9" max="9" width="15.625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11.625" customWidth="1"/>
     <col min="11" max="11" width="13.75" customWidth="1"/>
+    <col min="16" max="16" width="7.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:29" x14ac:dyDescent="0.25">
-      <c r="C1" s="6" t="s">
+    <row r="1" spans="3:23" x14ac:dyDescent="0.25">
+      <c r="C1" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
-      <c r="J1" s="5"/>
-      <c r="K1" s="5"/>
-    </row>
-    <row r="2" spans="3:29" x14ac:dyDescent="0.25">
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="16"/>
-    </row>
-    <row r="3" spans="3:29" x14ac:dyDescent="0.25">
-      <c r="Q3" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="R3" s="5"/>
-      <c r="S3" s="5"/>
-      <c r="T3" s="5"/>
-      <c r="U3" s="5"/>
-      <c r="V3" s="21">
-        <v>46169</v>
-      </c>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="J1" s="23"/>
+      <c r="K1" s="23"/>
+    </row>
+    <row r="2" spans="3:23" x14ac:dyDescent="0.25">
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="11"/>
+    </row>
+    <row r="3" spans="3:23" x14ac:dyDescent="0.25">
+      <c r="O3" s="16"/>
+      <c r="P3" s="21"/>
+      <c r="Q3" s="21"/>
+      <c r="R3" s="21"/>
+      <c r="S3" s="21"/>
+      <c r="T3" s="21"/>
+      <c r="U3" s="21"/>
+      <c r="V3" s="21"/>
       <c r="W3" s="21"/>
-      <c r="X3" s="21"/>
-      <c r="Y3" s="21"/>
-      <c r="Z3" s="21"/>
-      <c r="AA3" s="21"/>
-      <c r="AB3" s="21"/>
-      <c r="AC3" s="21"/>
-    </row>
-    <row r="4" spans="3:29" x14ac:dyDescent="0.25">
-      <c r="C4" s="5" t="s">
+    </row>
+    <row r="4" spans="3:23" x14ac:dyDescent="0.25">
+      <c r="C4" s="20" t="str">
+        <f>IF(Project_Department="Tbilisi","ქ. თბილისი","ქ. ბათუმი")</f>
+        <v>ქ. ბათუმი</v>
+      </c>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="I4" s="20" t="str">
+        <f>DAY(Handover_Date)&amp;" "&amp;IFERROR(VLOOKUP(MONTH(Handover_Date),{1,"იანვარი";2,"თებერვალი";3,"მარტი";4,"აპრილი";5,"მაისი";6,"ივნისი";7,"ივლისი";8,"აგვისტო";9,"სექტემბერი";10,"ოქტომბერი";11,"ნოემბერი";12,"დეკემბერი"},2,FALSE),"")&amp;" "&amp;YEAR(Handover_Date)</f>
+        <v>0 იანვარი 1900</v>
+      </c>
+      <c r="J4" s="20"/>
+      <c r="K4" s="20"/>
+    </row>
+    <row r="6" spans="3:23" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="22" t="str">
+        <f>"ერთი მხრივ "&amp;Project_Counteragent_Entity_Type&amp;" "&amp;Project_Counteragent_Name&amp;" -  წარმოდგენილი დირექტორის"&amp;Project_Counteragent_Director_Genitive&amp;" სახით (შემდგომში დამკვეთი)."&amp;CHAR(10)&amp;"მისამართი :"&amp;Project_Counteragent_Address_Line_1&amp;" "&amp;Project_Counteragent_Address_Line_2&amp;CHAR(10)&amp;"საიდენტიფიკაციო კოდი: "&amp;Project_Counteragent_ID&amp;CHAR(10)&amp;CHAR(10)&amp;"მეორე მხრივ, "&amp;Project_Insider_Entity_Type&amp;" "&amp;Project_Insider_Name &amp; " წარმოდგენილი დირექტორის "&amp; Project_Insider_Director_Genitive&amp;" სახით (შემდგომში შემსრულებელი)." &amp;CHAR(10)&amp;"მისამართი: "&amp;Project_Insider_Address_Line1&amp;" "&amp;Project_Insider_Address_Line2&amp;CHAR(10)&amp;"საიდენტიფიკაციო ნომერი:  "&amp;Project_Insider_ID&amp;Project_Insider_Entity_Type&amp;"."&amp;CHAR(10)&amp;CHAR(10)&amp;" ვადგენთ წინამდებარე აქტს მასზედ, რომ"&amp;IFERROR(YEAR(Contract_Date)&amp;" წლის "&amp;DAY(Contract_Date)&amp;" "&amp;VLOOKUP(MONTH(Contract_Date),{1,"იანვარის";2,"თებერვალის";3,"მარტის";4,"აპრილის";5,"მაისის";6,"ივნისის";7,"ივლისის";8,"აგვისტოს";9,"სექტემბრის";10,"ოქტომბრის";11,"ნოემბრის";12,"დეკემბრის"},2,FALSE),"")&amp;" ხელშეკრულების თანახმად დამკვეთმა მიიღო, ხოლო შემსრულებელმა ჩააბარა ქვემოთ მოცემული ლიფტები მისამართზე - "&amp;Project_Address&amp;" :"</f>
+        <v>ერთი მხრივ   -  წარმოდგენილი დირექტორის სახით (შემდგომში დამკვეთი).
+მისამართი : 
+საიდენტიფიკაციო კოდი: 
+მეორე მხრივ,   წარმოდგენილი დირექტორის  სახით (შემდგომში შემსრულებელი).
+მისამართი:  
+საიდენტიფიკაციო ნომერი:  .
+ ვადგენთ წინამდებარე აქტს მასზედ, რომ1900 წლის 0 იანვარის ხელშეკრულების თანახმად დამკვეთმა მიიღო, ხოლო შემსრულებელმა ჩააბარა ქვემოთ მოცემული ლიფტები მისამართზე -  :</v>
+      </c>
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="22"/>
+      <c r="I6" s="22"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="22"/>
+    </row>
+    <row r="7" spans="3:23" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C7" s="22"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="22"/>
+      <c r="I7" s="22"/>
+      <c r="J7" s="22"/>
+      <c r="K7" s="22"/>
+    </row>
+    <row r="8" spans="3:23" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="22"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="22"/>
+      <c r="I8" s="22"/>
+      <c r="J8" s="22"/>
+      <c r="K8" s="22"/>
+    </row>
+    <row r="9" spans="3:23" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="22"/>
+      <c r="I9" s="22"/>
+      <c r="J9" s="22"/>
+      <c r="K9" s="22"/>
+    </row>
+    <row r="10" spans="3:23" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="22"/>
+      <c r="I10" s="22"/>
+      <c r="J10" s="22"/>
+      <c r="K10" s="22"/>
+    </row>
+    <row r="11" spans="3:23" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
+      <c r="G11" s="22"/>
+      <c r="H11" s="22"/>
+      <c r="I11" s="22"/>
+      <c r="J11" s="22"/>
+      <c r="K11" s="22"/>
+    </row>
+    <row r="12" spans="3:23" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="22"/>
+      <c r="H12" s="22"/>
+      <c r="I12" s="22"/>
+      <c r="J12" s="22"/>
+      <c r="K12" s="22"/>
+    </row>
+    <row r="13" spans="3:23" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
+      <c r="G13" s="22"/>
+      <c r="H13" s="22"/>
+      <c r="I13" s="22"/>
+      <c r="J13" s="22"/>
+      <c r="K13" s="22"/>
+    </row>
+    <row r="14" spans="3:23" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
+      <c r="G14" s="22"/>
+      <c r="H14" s="22"/>
+      <c r="I14" s="22"/>
+      <c r="J14" s="22"/>
+      <c r="K14" s="22"/>
+    </row>
+    <row r="16" spans="3:23" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="C16" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="J4" s="5" t="s">
+      <c r="D16" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="F16" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="H16" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="K4" s="5"/>
-    </row>
-    <row r="6" spans="3:29" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C6" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
-    </row>
-    <row r="7" spans="3:29" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-    </row>
-    <row r="8" spans="3:29" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="9"/>
-    </row>
-    <row r="9" spans="3:29" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
-    </row>
-    <row r="10" spans="3:29" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
-      <c r="K10" s="9"/>
-    </row>
-    <row r="11" spans="3:29" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="9"/>
-    </row>
-    <row r="12" spans="3:29" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-    </row>
-    <row r="13" spans="3:29" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
-      <c r="K13" s="9"/>
-    </row>
-    <row r="14" spans="3:29" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
-      <c r="K14" s="9"/>
-    </row>
-    <row r="16" spans="3:29" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="C16" s="10" t="s">
+      <c r="I16" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="J16" s="6" t="str">
+        <f>"თანხა "&amp;IF(Project_Currency="USD"," $", IF(Project_Currency = "EUR", " €"," ₾"))</f>
+        <v>თანხა  ₾</v>
+      </c>
+      <c r="K16" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="D16" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="E16" s="10" t="s">
+    </row>
+    <row r="17" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C17" s="7" t="e" vm="1">
+        <f ca="1">IF(D17&lt;&gt;"",ROW()-16,"")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D17" s="7" t="e" cm="1" vm="2">
+        <f t="array" aca="1" ref="D17" ca="1">_xlfn._xlws.FILTER(Jobs!A:A,Jobs!M:M= Handover_Date)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E17" s="7" t="e" cm="1" vm="2">
+        <f t="array" aca="1" ref="E17" ca="1">_xlfn._xlws.FILTER( Jobs!C:C,Jobs!M:M= Handover_Date)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="F17" s="7" t="e" cm="1" vm="2">
+        <f t="array" aca="1" ref="F17" ca="1">_xlfn._xlws.FILTER(   Jobs!B:B,Jobs!M:M= Handover_Date)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="G17" s="7" t="e" cm="1" vm="2">
+        <f t="array" aca="1" ref="G17" ca="1">_xlfn._xlws.FILTER(  Jobs!E:E,Jobs!M:M= Handover_Date)&amp;" კგ"</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="H17" s="7" t="e" cm="1" vm="2">
+        <f t="array" aca="1" ref="H17" ca="1">_xlfn._xlws.FILTER(   Jobs!D:D,Jobs!M:M= Handover_Date)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="I17" s="7" t="e" cm="1" vm="2">
+        <f t="array" aca="1" ref="I17" ca="1">_xlfn._xlws.FILTER(    Jobs!N:N,Jobs!M:M= Handover_Date)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="J17" s="8" t="e" cm="1" vm="2">
+        <f t="array" aca="1" ref="J17" ca="1">_xlfn._xlws.FILTER(    Jobs!F:F,Jobs!M:M= Handover_Date)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="K17" s="8" t="e" cm="1" vm="2">
+        <f t="array" aca="1" ref="K17" ca="1">_xlfn._xlws.FILTER(     Jobs!K:K,Jobs!M:M= Handover_Date)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="18" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C18" s="7" t="str">
+        <f t="shared" ref="C18:C63" si="0">IF(D18&lt;&gt;"",ROW()-16,"")</f>
+        <v/>
+      </c>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="7"/>
+      <c r="J18" s="8"/>
+      <c r="K18" s="8"/>
+    </row>
+    <row r="19" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C19" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="7"/>
+      <c r="J19" s="8"/>
+      <c r="K19" s="8"/>
+    </row>
+    <row r="20" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C20" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="7"/>
+      <c r="H20" s="7"/>
+      <c r="I20" s="7"/>
+      <c r="J20" s="8"/>
+      <c r="K20" s="8"/>
+    </row>
+    <row r="21" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C21" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="7"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="7"/>
+      <c r="J21" s="8"/>
+      <c r="K21" s="8"/>
+    </row>
+    <row r="22" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C22" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="7"/>
+      <c r="J22" s="8"/>
+      <c r="K22" s="8"/>
+    </row>
+    <row r="23" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C23" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
+      <c r="H23" s="7"/>
+      <c r="I23" s="7"/>
+      <c r="J23" s="8"/>
+      <c r="K23" s="8"/>
+    </row>
+    <row r="24" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C24" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="7"/>
+      <c r="G24" s="7"/>
+      <c r="H24" s="7"/>
+      <c r="I24" s="7"/>
+      <c r="J24" s="8"/>
+      <c r="K24" s="8"/>
+    </row>
+    <row r="25" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C25" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
+      <c r="H25" s="7"/>
+      <c r="I25" s="7"/>
+      <c r="J25" s="8"/>
+      <c r="K25" s="8"/>
+    </row>
+    <row r="26" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C26" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
+      <c r="F26" s="7"/>
+      <c r="G26" s="7"/>
+      <c r="H26" s="7"/>
+      <c r="I26" s="7"/>
+      <c r="J26" s="8"/>
+      <c r="K26" s="8"/>
+    </row>
+    <row r="27" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C27" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D27" s="7"/>
+      <c r="E27" s="7"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="7"/>
+      <c r="H27" s="7"/>
+      <c r="I27" s="7"/>
+      <c r="J27" s="8"/>
+      <c r="K27" s="8"/>
+    </row>
+    <row r="28" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C28" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D28" s="7"/>
+      <c r="E28" s="7"/>
+      <c r="F28" s="7"/>
+      <c r="G28" s="7"/>
+      <c r="H28" s="7"/>
+      <c r="I28" s="7"/>
+      <c r="J28" s="8"/>
+      <c r="K28" s="8"/>
+    </row>
+    <row r="29" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C29" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D29" s="7"/>
+      <c r="E29" s="7"/>
+      <c r="F29" s="7"/>
+      <c r="G29" s="7"/>
+      <c r="H29" s="7"/>
+      <c r="I29" s="7"/>
+      <c r="J29" s="8"/>
+      <c r="K29" s="8"/>
+    </row>
+    <row r="30" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C30" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D30" s="7"/>
+      <c r="E30" s="7"/>
+      <c r="F30" s="7"/>
+      <c r="G30" s="7"/>
+      <c r="H30" s="7"/>
+      <c r="I30" s="7"/>
+      <c r="J30" s="8"/>
+      <c r="K30" s="8"/>
+    </row>
+    <row r="31" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C31" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
+      <c r="F31" s="7"/>
+      <c r="G31" s="7"/>
+      <c r="H31" s="7"/>
+      <c r="I31" s="7"/>
+      <c r="J31" s="8"/>
+      <c r="K31" s="8"/>
+    </row>
+    <row r="32" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C32" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D32" s="7"/>
+      <c r="E32" s="7"/>
+      <c r="F32" s="7"/>
+      <c r="G32" s="7"/>
+      <c r="H32" s="7"/>
+      <c r="I32" s="7"/>
+      <c r="J32" s="8"/>
+      <c r="K32" s="8"/>
+    </row>
+    <row r="33" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C33" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D33" s="7"/>
+      <c r="E33" s="7"/>
+      <c r="F33" s="7"/>
+      <c r="G33" s="7"/>
+      <c r="H33" s="7"/>
+      <c r="I33" s="7"/>
+      <c r="J33" s="8"/>
+      <c r="K33" s="8"/>
+    </row>
+    <row r="34" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C34" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D34" s="7"/>
+      <c r="E34" s="7"/>
+      <c r="F34" s="7"/>
+      <c r="G34" s="7"/>
+      <c r="H34" s="7"/>
+      <c r="I34" s="7"/>
+      <c r="J34" s="8"/>
+      <c r="K34" s="8"/>
+    </row>
+    <row r="35" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C35" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D35" s="7"/>
+      <c r="E35" s="7"/>
+      <c r="F35" s="7"/>
+      <c r="G35" s="7"/>
+      <c r="H35" s="7"/>
+      <c r="I35" s="7"/>
+      <c r="J35" s="8"/>
+      <c r="K35" s="8"/>
+    </row>
+    <row r="36" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C36" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D36" s="7"/>
+      <c r="E36" s="7"/>
+      <c r="F36" s="7"/>
+      <c r="G36" s="7"/>
+      <c r="H36" s="7"/>
+      <c r="I36" s="7"/>
+      <c r="J36" s="8"/>
+      <c r="K36" s="8"/>
+    </row>
+    <row r="37" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C37" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D37" s="7"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="7"/>
+      <c r="G37" s="7"/>
+      <c r="H37" s="7"/>
+      <c r="I37" s="7"/>
+      <c r="J37" s="8"/>
+      <c r="K37" s="8"/>
+    </row>
+    <row r="38" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C38" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D38" s="7"/>
+      <c r="E38" s="7"/>
+      <c r="F38" s="7"/>
+      <c r="G38" s="7"/>
+      <c r="H38" s="7"/>
+      <c r="I38" s="7"/>
+      <c r="J38" s="8"/>
+      <c r="K38" s="8"/>
+    </row>
+    <row r="39" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C39" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D39" s="7"/>
+      <c r="E39" s="7"/>
+      <c r="F39" s="7"/>
+      <c r="G39" s="7"/>
+      <c r="H39" s="7"/>
+      <c r="I39" s="7"/>
+      <c r="J39" s="8"/>
+      <c r="K39" s="8"/>
+    </row>
+    <row r="40" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C40" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D40" s="7"/>
+      <c r="E40" s="7"/>
+      <c r="F40" s="7"/>
+      <c r="G40" s="7"/>
+      <c r="H40" s="7"/>
+      <c r="I40" s="7"/>
+      <c r="J40" s="8"/>
+      <c r="K40" s="8"/>
+    </row>
+    <row r="41" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C41" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D41" s="7"/>
+      <c r="E41" s="7"/>
+      <c r="F41" s="7"/>
+      <c r="G41" s="7"/>
+      <c r="H41" s="7"/>
+      <c r="I41" s="7"/>
+      <c r="J41" s="8"/>
+      <c r="K41" s="8"/>
+    </row>
+    <row r="42" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C42" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D42" s="7"/>
+      <c r="E42" s="7"/>
+      <c r="F42" s="7"/>
+      <c r="G42" s="7"/>
+      <c r="H42" s="7"/>
+      <c r="I42" s="7"/>
+      <c r="J42" s="8"/>
+      <c r="K42" s="8"/>
+    </row>
+    <row r="43" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C43" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D43" s="7"/>
+      <c r="E43" s="7"/>
+      <c r="F43" s="7"/>
+      <c r="G43" s="7"/>
+      <c r="H43" s="7"/>
+      <c r="I43" s="7"/>
+      <c r="J43" s="8"/>
+      <c r="K43" s="8"/>
+    </row>
+    <row r="44" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C44" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D44" s="7"/>
+      <c r="E44" s="7"/>
+      <c r="F44" s="7"/>
+      <c r="G44" s="7"/>
+      <c r="H44" s="7"/>
+      <c r="I44" s="7"/>
+      <c r="J44" s="8"/>
+      <c r="K44" s="8"/>
+    </row>
+    <row r="45" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C45" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D45" s="7"/>
+      <c r="E45" s="7"/>
+      <c r="F45" s="7"/>
+      <c r="G45" s="7"/>
+      <c r="H45" s="7"/>
+      <c r="I45" s="7"/>
+      <c r="J45" s="8"/>
+      <c r="K45" s="8"/>
+    </row>
+    <row r="46" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C46" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D46" s="7"/>
+      <c r="E46" s="7"/>
+      <c r="F46" s="7"/>
+      <c r="G46" s="7"/>
+      <c r="H46" s="7"/>
+      <c r="I46" s="7"/>
+      <c r="J46" s="8"/>
+      <c r="K46" s="8"/>
+    </row>
+    <row r="47" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C47" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D47" s="7"/>
+      <c r="E47" s="7"/>
+      <c r="F47" s="7"/>
+      <c r="G47" s="7"/>
+      <c r="H47" s="7"/>
+      <c r="I47" s="7"/>
+      <c r="J47" s="8"/>
+      <c r="K47" s="8"/>
+    </row>
+    <row r="48" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C48" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D48" s="7"/>
+      <c r="E48" s="7"/>
+      <c r="F48" s="7"/>
+      <c r="G48" s="7"/>
+      <c r="H48" s="7"/>
+      <c r="I48" s="7"/>
+      <c r="J48" s="8"/>
+      <c r="K48" s="8"/>
+    </row>
+    <row r="49" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C49" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D49" s="7"/>
+      <c r="E49" s="7"/>
+      <c r="F49" s="7"/>
+      <c r="G49" s="7"/>
+      <c r="H49" s="7"/>
+      <c r="I49" s="7"/>
+      <c r="J49" s="8"/>
+      <c r="K49" s="8"/>
+    </row>
+    <row r="50" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C50" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D50" s="7"/>
+      <c r="E50" s="7"/>
+      <c r="F50" s="7"/>
+      <c r="G50" s="7"/>
+      <c r="H50" s="7"/>
+      <c r="I50" s="7"/>
+      <c r="J50" s="8"/>
+      <c r="K50" s="8"/>
+    </row>
+    <row r="51" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C51" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D51" s="7"/>
+      <c r="E51" s="7"/>
+      <c r="F51" s="7"/>
+      <c r="G51" s="7"/>
+      <c r="H51" s="7"/>
+      <c r="I51" s="7"/>
+      <c r="J51" s="8"/>
+      <c r="K51" s="8"/>
+    </row>
+    <row r="52" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C52" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D52" s="7"/>
+      <c r="E52" s="7"/>
+      <c r="F52" s="7"/>
+      <c r="G52" s="7"/>
+      <c r="H52" s="7"/>
+      <c r="I52" s="7"/>
+      <c r="J52" s="8"/>
+      <c r="K52" s="8"/>
+    </row>
+    <row r="53" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C53" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D53" s="7"/>
+      <c r="E53" s="7"/>
+      <c r="F53" s="7"/>
+      <c r="G53" s="7"/>
+      <c r="H53" s="7"/>
+      <c r="I53" s="7"/>
+      <c r="J53" s="8"/>
+      <c r="K53" s="8"/>
+    </row>
+    <row r="54" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C54" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D54" s="7"/>
+      <c r="E54" s="7"/>
+      <c r="F54" s="7"/>
+      <c r="G54" s="7"/>
+      <c r="H54" s="7"/>
+      <c r="I54" s="7"/>
+      <c r="J54" s="8"/>
+      <c r="K54" s="8"/>
+    </row>
+    <row r="55" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C55" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D55" s="7"/>
+      <c r="E55" s="7"/>
+      <c r="F55" s="7"/>
+      <c r="G55" s="7"/>
+      <c r="H55" s="7"/>
+      <c r="I55" s="7"/>
+      <c r="J55" s="8"/>
+      <c r="K55" s="8"/>
+    </row>
+    <row r="56" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C56" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D56" s="7"/>
+      <c r="E56" s="7"/>
+      <c r="F56" s="7"/>
+      <c r="G56" s="7"/>
+      <c r="H56" s="7"/>
+      <c r="I56" s="7"/>
+      <c r="J56" s="8"/>
+      <c r="K56" s="8"/>
+    </row>
+    <row r="57" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C57" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D57" s="7"/>
+      <c r="E57" s="7"/>
+      <c r="F57" s="7"/>
+      <c r="G57" s="7"/>
+      <c r="H57" s="7"/>
+      <c r="I57" s="7"/>
+      <c r="J57" s="8"/>
+      <c r="K57" s="8"/>
+    </row>
+    <row r="58" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C58" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D58" s="7"/>
+      <c r="E58" s="7"/>
+      <c r="F58" s="7"/>
+      <c r="G58" s="7"/>
+      <c r="H58" s="7"/>
+      <c r="I58" s="7"/>
+      <c r="J58" s="8"/>
+      <c r="K58" s="8"/>
+    </row>
+    <row r="59" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C59" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D59" s="7"/>
+      <c r="E59" s="7"/>
+      <c r="F59" s="7"/>
+      <c r="G59" s="7"/>
+      <c r="H59" s="7"/>
+      <c r="I59" s="7"/>
+      <c r="J59" s="8"/>
+      <c r="K59" s="8"/>
+    </row>
+    <row r="60" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C60" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D60" s="7"/>
+      <c r="E60" s="7"/>
+      <c r="F60" s="7"/>
+      <c r="G60" s="7"/>
+      <c r="H60" s="7"/>
+      <c r="I60" s="7"/>
+      <c r="J60" s="8"/>
+      <c r="K60" s="8"/>
+    </row>
+    <row r="61" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C61" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D61" s="7"/>
+      <c r="E61" s="7"/>
+      <c r="F61" s="7"/>
+      <c r="G61" s="7"/>
+      <c r="H61" s="7"/>
+      <c r="I61" s="7"/>
+      <c r="J61" s="8"/>
+      <c r="K61" s="8"/>
+    </row>
+    <row r="62" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C62" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D62" s="7"/>
+      <c r="E62" s="7"/>
+      <c r="F62" s="7"/>
+      <c r="G62" s="7"/>
+      <c r="H62" s="7"/>
+      <c r="I62" s="7"/>
+      <c r="J62" s="8"/>
+      <c r="K62" s="8"/>
+    </row>
+    <row r="63" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C63" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="D63" s="7"/>
+      <c r="E63" s="7"/>
+      <c r="F63" s="7"/>
+      <c r="G63" s="7"/>
+      <c r="H63" s="7"/>
+      <c r="I63" s="7"/>
+      <c r="J63" s="8"/>
+      <c r="K63" s="8"/>
+    </row>
+    <row r="64" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C64" s="19" t="s">
         <v>79</v>
       </c>
-      <c r="F16" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="G16" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="H16" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="I16" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="J16" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="K16" s="10" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="17" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C17" s="11">
-        <f>IF(D17&lt;&gt;"",ROW()-16,"")</f>
-        <v>1</v>
-      </c>
-      <c r="D17" s="11" t="str" cm="1">
-        <f t="array" ref="D17:D18">_xlfn._xlws.FILTER(Jobs!A:A,Jobs!M:M= V3)</f>
-        <v>L0001</v>
-      </c>
-      <c r="E17" s="11" t="str" cm="1">
-        <f t="array" ref="E17:E18">_xlfn._xlws.FILTER( Jobs!C:C,Jobs!M:M= V3)</f>
-        <v>OTIS</v>
-      </c>
-      <c r="F17" s="11" t="str" cm="1">
-        <f t="array" ref="F17:F18">_xlfn._xlws.FILTER(   Jobs!B:B,Jobs!M:M= V3)</f>
-        <v>K6NC0632</v>
-      </c>
-      <c r="G17" s="11" t="str" cm="1">
-        <f t="array" ref="G17:G18">_xlfn._xlws.FILTER(  Jobs!E:E,Jobs!M:M= V3)&amp;" კგ"</f>
-        <v>1000 კგ</v>
-      </c>
-      <c r="H17" s="11" cm="1">
-        <f t="array" ref="H17:H18">_xlfn._xlws.FILTER(   Jobs!D:D,Jobs!M:M= V3)</f>
-        <v>13</v>
-      </c>
-      <c r="I17" s="11" t="str" cm="1">
-        <f t="array" ref="I17:I18">_xlfn._xlws.FILTER(    Jobs!N:N,Jobs!M:M= V3)</f>
-        <v>0860-26</v>
-      </c>
-      <c r="J17" s="12" cm="1">
-        <f t="array" ref="J17:J18">_xlfn._xlws.FILTER(    Jobs!F:F,Jobs!M:M= V3)</f>
-        <v>44088</v>
-      </c>
-      <c r="K17" s="12" cm="1">
-        <f t="array" ref="K17:K18">_xlfn._xlws.FILTER(     Jobs!K:K,Jobs!M:M= V3)</f>
-        <v>118268.1</v>
-      </c>
-    </row>
-    <row r="18" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C18" s="11">
-        <f t="shared" ref="C18:C63" si="0">IF(D18&lt;&gt;"",ROW()-16,"")</f>
-        <v>2</v>
-      </c>
-      <c r="D18" s="11" t="str">
-        <v>L0002</v>
-      </c>
-      <c r="E18" s="11" t="str">
-        <v>OTIS</v>
-      </c>
-      <c r="F18" s="11" t="str">
-        <v>K6NC0633</v>
-      </c>
-      <c r="G18" s="11" t="str">
-        <v>1600 კგ</v>
-      </c>
-      <c r="H18" s="11">
-        <v>13</v>
-      </c>
-      <c r="I18" s="11" t="str">
-        <v>0861-26</v>
-      </c>
-      <c r="J18" s="12">
-        <v>55044</v>
-      </c>
-      <c r="K18" s="12">
-        <v>147664.18</v>
-      </c>
-    </row>
-    <row r="19" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C19" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="11"/>
-      <c r="J19" s="12"/>
-      <c r="K19" s="12"/>
-    </row>
-    <row r="20" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C20" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="11"/>
-      <c r="J20" s="12"/>
-      <c r="K20" s="12"/>
-    </row>
-    <row r="21" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C21" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="11"/>
-      <c r="J21" s="12"/>
-      <c r="K21" s="12"/>
-    </row>
-    <row r="22" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C22" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="11"/>
-      <c r="J22" s="12"/>
-      <c r="K22" s="12"/>
-    </row>
-    <row r="23" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C23" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="11"/>
-      <c r="I23" s="11"/>
-      <c r="J23" s="12"/>
-      <c r="K23" s="12"/>
-    </row>
-    <row r="24" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C24" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="11"/>
-      <c r="H24" s="11"/>
-      <c r="I24" s="11"/>
-      <c r="J24" s="12"/>
-      <c r="K24" s="12"/>
-    </row>
-    <row r="25" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C25" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="11"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="11"/>
-      <c r="J25" s="12"/>
-      <c r="K25" s="12"/>
-    </row>
-    <row r="26" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C26" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="11"/>
-      <c r="H26" s="11"/>
-      <c r="I26" s="11"/>
-      <c r="J26" s="12"/>
-      <c r="K26" s="12"/>
-    </row>
-    <row r="27" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C27" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D27" s="11"/>
-      <c r="E27" s="11"/>
-      <c r="F27" s="11"/>
-      <c r="G27" s="11"/>
-      <c r="H27" s="11"/>
-      <c r="I27" s="11"/>
-      <c r="J27" s="12"/>
-      <c r="K27" s="12"/>
-    </row>
-    <row r="28" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C28" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D28" s="11"/>
-      <c r="E28" s="11"/>
-      <c r="F28" s="11"/>
-      <c r="G28" s="11"/>
-      <c r="H28" s="11"/>
-      <c r="I28" s="11"/>
-      <c r="J28" s="12"/>
-      <c r="K28" s="12"/>
-    </row>
-    <row r="29" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C29" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D29" s="11"/>
-      <c r="E29" s="11"/>
-      <c r="F29" s="11"/>
-      <c r="G29" s="11"/>
-      <c r="H29" s="11"/>
-      <c r="I29" s="11"/>
-      <c r="J29" s="12"/>
-      <c r="K29" s="12"/>
-    </row>
-    <row r="30" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C30" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D30" s="11"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="11"/>
-      <c r="G30" s="11"/>
-      <c r="H30" s="11"/>
-      <c r="I30" s="11"/>
-      <c r="J30" s="12"/>
-      <c r="K30" s="12"/>
-    </row>
-    <row r="31" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C31" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D31" s="11"/>
-      <c r="E31" s="11"/>
-      <c r="F31" s="11"/>
-      <c r="G31" s="11"/>
-      <c r="H31" s="11"/>
-      <c r="I31" s="11"/>
-      <c r="J31" s="12"/>
-      <c r="K31" s="12"/>
-    </row>
-    <row r="32" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C32" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D32" s="11"/>
-      <c r="E32" s="11"/>
-      <c r="F32" s="11"/>
-      <c r="G32" s="11"/>
-      <c r="H32" s="11"/>
-      <c r="I32" s="11"/>
-      <c r="J32" s="12"/>
-      <c r="K32" s="12"/>
-    </row>
-    <row r="33" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C33" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D33" s="11"/>
-      <c r="E33" s="11"/>
-      <c r="F33" s="11"/>
-      <c r="G33" s="11"/>
-      <c r="H33" s="11"/>
-      <c r="I33" s="11"/>
-      <c r="J33" s="12"/>
-      <c r="K33" s="12"/>
-    </row>
-    <row r="34" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C34" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D34" s="11"/>
-      <c r="E34" s="11"/>
-      <c r="F34" s="11"/>
-      <c r="G34" s="11"/>
-      <c r="H34" s="11"/>
-      <c r="I34" s="11"/>
-      <c r="J34" s="12"/>
-      <c r="K34" s="12"/>
-    </row>
-    <row r="35" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C35" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D35" s="11"/>
-      <c r="E35" s="11"/>
-      <c r="F35" s="11"/>
-      <c r="G35" s="11"/>
-      <c r="H35" s="11"/>
-      <c r="I35" s="11"/>
-      <c r="J35" s="12"/>
-      <c r="K35" s="12"/>
-    </row>
-    <row r="36" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C36" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D36" s="11"/>
-      <c r="E36" s="11"/>
-      <c r="F36" s="11"/>
-      <c r="G36" s="11"/>
-      <c r="H36" s="11"/>
-      <c r="I36" s="11"/>
-      <c r="J36" s="12"/>
-      <c r="K36" s="12"/>
-    </row>
-    <row r="37" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C37" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D37" s="11"/>
-      <c r="E37" s="11"/>
-      <c r="F37" s="11"/>
-      <c r="G37" s="11"/>
-      <c r="H37" s="11"/>
-      <c r="I37" s="11"/>
-      <c r="J37" s="12"/>
-      <c r="K37" s="12"/>
-    </row>
-    <row r="38" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C38" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D38" s="11"/>
-      <c r="E38" s="11"/>
-      <c r="F38" s="11"/>
-      <c r="G38" s="11"/>
-      <c r="H38" s="11"/>
-      <c r="I38" s="11"/>
-      <c r="J38" s="12"/>
-      <c r="K38" s="12"/>
-    </row>
-    <row r="39" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C39" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D39" s="11"/>
-      <c r="E39" s="11"/>
-      <c r="F39" s="11"/>
-      <c r="G39" s="11"/>
-      <c r="H39" s="11"/>
-      <c r="I39" s="11"/>
-      <c r="J39" s="12"/>
-      <c r="K39" s="12"/>
-    </row>
-    <row r="40" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C40" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D40" s="11"/>
-      <c r="E40" s="11"/>
-      <c r="F40" s="11"/>
-      <c r="G40" s="11"/>
-      <c r="H40" s="11"/>
-      <c r="I40" s="11"/>
-      <c r="J40" s="12"/>
-      <c r="K40" s="12"/>
-    </row>
-    <row r="41" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C41" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D41" s="11"/>
-      <c r="E41" s="11"/>
-      <c r="F41" s="11"/>
-      <c r="G41" s="11"/>
-      <c r="H41" s="11"/>
-      <c r="I41" s="11"/>
-      <c r="J41" s="12"/>
-      <c r="K41" s="12"/>
-    </row>
-    <row r="42" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C42" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D42" s="11"/>
-      <c r="E42" s="11"/>
-      <c r="F42" s="11"/>
-      <c r="G42" s="11"/>
-      <c r="H42" s="11"/>
-      <c r="I42" s="11"/>
-      <c r="J42" s="12"/>
-      <c r="K42" s="12"/>
-    </row>
-    <row r="43" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C43" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D43" s="11"/>
-      <c r="E43" s="11"/>
-      <c r="F43" s="11"/>
-      <c r="G43" s="11"/>
-      <c r="H43" s="11"/>
-      <c r="I43" s="11"/>
-      <c r="J43" s="12"/>
-      <c r="K43" s="12"/>
-    </row>
-    <row r="44" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C44" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D44" s="11"/>
-      <c r="E44" s="11"/>
-      <c r="F44" s="11"/>
-      <c r="G44" s="11"/>
-      <c r="H44" s="11"/>
-      <c r="I44" s="11"/>
-      <c r="J44" s="12"/>
-      <c r="K44" s="12"/>
-    </row>
-    <row r="45" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C45" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D45" s="11"/>
-      <c r="E45" s="11"/>
-      <c r="F45" s="11"/>
-      <c r="G45" s="11"/>
-      <c r="H45" s="11"/>
-      <c r="I45" s="11"/>
-      <c r="J45" s="12"/>
-      <c r="K45" s="12"/>
-    </row>
-    <row r="46" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C46" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D46" s="11"/>
-      <c r="E46" s="11"/>
-      <c r="F46" s="11"/>
-      <c r="G46" s="11"/>
-      <c r="H46" s="11"/>
-      <c r="I46" s="11"/>
-      <c r="J46" s="12"/>
-      <c r="K46" s="12"/>
-    </row>
-    <row r="47" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C47" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D47" s="11"/>
-      <c r="E47" s="11"/>
-      <c r="F47" s="11"/>
-      <c r="G47" s="11"/>
-      <c r="H47" s="11"/>
-      <c r="I47" s="11"/>
-      <c r="J47" s="12"/>
-      <c r="K47" s="12"/>
-    </row>
-    <row r="48" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C48" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D48" s="11"/>
-      <c r="E48" s="11"/>
-      <c r="F48" s="11"/>
-      <c r="G48" s="11"/>
-      <c r="H48" s="11"/>
-      <c r="I48" s="11"/>
-      <c r="J48" s="12"/>
-      <c r="K48" s="12"/>
-    </row>
-    <row r="49" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C49" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D49" s="11"/>
-      <c r="E49" s="11"/>
-      <c r="F49" s="11"/>
-      <c r="G49" s="11"/>
-      <c r="H49" s="11"/>
-      <c r="I49" s="11"/>
-      <c r="J49" s="12"/>
-      <c r="K49" s="12"/>
-    </row>
-    <row r="50" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C50" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D50" s="11"/>
-      <c r="E50" s="11"/>
-      <c r="F50" s="11"/>
-      <c r="G50" s="11"/>
-      <c r="H50" s="11"/>
-      <c r="I50" s="11"/>
-      <c r="J50" s="12"/>
-      <c r="K50" s="12"/>
-    </row>
-    <row r="51" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C51" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D51" s="11"/>
-      <c r="E51" s="11"/>
-      <c r="F51" s="11"/>
-      <c r="G51" s="11"/>
-      <c r="H51" s="11"/>
-      <c r="I51" s="11"/>
-      <c r="J51" s="12"/>
-      <c r="K51" s="12"/>
-    </row>
-    <row r="52" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C52" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D52" s="11"/>
-      <c r="E52" s="11"/>
-      <c r="F52" s="11"/>
-      <c r="G52" s="11"/>
-      <c r="H52" s="11"/>
-      <c r="I52" s="11"/>
-      <c r="J52" s="12"/>
-      <c r="K52" s="12"/>
-    </row>
-    <row r="53" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C53" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D53" s="11"/>
-      <c r="E53" s="11"/>
-      <c r="F53" s="11"/>
-      <c r="G53" s="11"/>
-      <c r="H53" s="11"/>
-      <c r="I53" s="11"/>
-      <c r="J53" s="12"/>
-      <c r="K53" s="12"/>
-    </row>
-    <row r="54" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C54" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D54" s="11"/>
-      <c r="E54" s="11"/>
-      <c r="F54" s="11"/>
-      <c r="G54" s="11"/>
-      <c r="H54" s="11"/>
-      <c r="I54" s="11"/>
-      <c r="J54" s="12"/>
-      <c r="K54" s="12"/>
-    </row>
-    <row r="55" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C55" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D55" s="11"/>
-      <c r="E55" s="11"/>
-      <c r="F55" s="11"/>
-      <c r="G55" s="11"/>
-      <c r="H55" s="11"/>
-      <c r="I55" s="11"/>
-      <c r="J55" s="12"/>
-      <c r="K55" s="12"/>
-    </row>
-    <row r="56" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C56" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D56" s="11"/>
-      <c r="E56" s="11"/>
-      <c r="F56" s="11"/>
-      <c r="G56" s="11"/>
-      <c r="H56" s="11"/>
-      <c r="I56" s="11"/>
-      <c r="J56" s="12"/>
-      <c r="K56" s="12"/>
-    </row>
-    <row r="57" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C57" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D57" s="11"/>
-      <c r="E57" s="11"/>
-      <c r="F57" s="11"/>
-      <c r="G57" s="11"/>
-      <c r="H57" s="11"/>
-      <c r="I57" s="11"/>
-      <c r="J57" s="12"/>
-      <c r="K57" s="12"/>
-    </row>
-    <row r="58" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C58" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D58" s="11"/>
-      <c r="E58" s="11"/>
-      <c r="F58" s="11"/>
-      <c r="G58" s="11"/>
-      <c r="H58" s="11"/>
-      <c r="I58" s="11"/>
-      <c r="J58" s="12"/>
-      <c r="K58" s="12"/>
-    </row>
-    <row r="59" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C59" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D59" s="11"/>
-      <c r="E59" s="11"/>
-      <c r="F59" s="11"/>
-      <c r="G59" s="11"/>
-      <c r="H59" s="11"/>
-      <c r="I59" s="11"/>
-      <c r="J59" s="12"/>
-      <c r="K59" s="12"/>
-    </row>
-    <row r="60" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C60" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D60" s="11"/>
-      <c r="E60" s="11"/>
-      <c r="F60" s="11"/>
-      <c r="G60" s="11"/>
-      <c r="H60" s="11"/>
-      <c r="I60" s="11"/>
-      <c r="J60" s="12"/>
-      <c r="K60" s="12"/>
-    </row>
-    <row r="61" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C61" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D61" s="11"/>
-      <c r="E61" s="11"/>
-      <c r="F61" s="11"/>
-      <c r="G61" s="11"/>
-      <c r="H61" s="11"/>
-      <c r="I61" s="11"/>
-      <c r="J61" s="12"/>
-      <c r="K61" s="12"/>
-    </row>
-    <row r="62" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C62" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D62" s="11"/>
-      <c r="E62" s="11"/>
-      <c r="F62" s="11"/>
-      <c r="G62" s="11"/>
-      <c r="H62" s="11"/>
-      <c r="I62" s="11"/>
-      <c r="J62" s="12"/>
-      <c r="K62" s="12"/>
-    </row>
-    <row r="63" spans="3:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C63" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D63" s="11"/>
-      <c r="E63" s="11"/>
-      <c r="F63" s="11"/>
-      <c r="G63" s="11"/>
-      <c r="H63" s="11"/>
-      <c r="I63" s="11"/>
-      <c r="J63" s="12"/>
-      <c r="K63" s="12"/>
-    </row>
-    <row r="64" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C64" s="13" t="s">
-        <v>83</v>
-      </c>
-      <c r="D64" s="13"/>
-      <c r="E64" s="13"/>
-      <c r="F64" s="13"/>
-      <c r="G64" s="13"/>
-      <c r="H64" s="13"/>
-      <c r="I64" s="11"/>
-      <c r="J64" s="12">
-        <f>SUM(J17:J63)</f>
-        <v>99132</v>
-      </c>
-      <c r="K64" s="12">
-        <f>SUM(K17:K63)</f>
-        <v>265932.28000000003</v>
+      <c r="D64" s="19"/>
+      <c r="E64" s="19"/>
+      <c r="F64" s="19"/>
+      <c r="G64" s="19"/>
+      <c r="H64" s="19"/>
+      <c r="I64" s="7"/>
+      <c r="J64" s="8" t="e" vm="1">
+        <f ca="1">SUM(J17:J63)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="K64" s="8" t="e" vm="1">
+        <f ca="1">SUM(K17:K63)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="65" spans="3:12" x14ac:dyDescent="0.25">
@@ -1748,17 +1894,17 @@
       <c r="D65" s="4"/>
     </row>
     <row r="66" spans="3:12" ht="139.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C66" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="D66" s="18"/>
-      <c r="E66" s="18"/>
-      <c r="F66" s="18"/>
-      <c r="G66" s="18"/>
-      <c r="H66" s="18"/>
-      <c r="I66" s="18"/>
-      <c r="J66" s="18"/>
-      <c r="K66" s="18"/>
+      <c r="C66" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="D66" s="25"/>
+      <c r="E66" s="25"/>
+      <c r="F66" s="25"/>
+      <c r="G66" s="25"/>
+      <c r="H66" s="25"/>
+      <c r="I66" s="25"/>
+      <c r="J66" s="25"/>
+      <c r="K66" s="25"/>
     </row>
     <row r="67" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C67" s="4"/>
@@ -1769,140 +1915,150 @@
       <c r="D68" s="4"/>
     </row>
     <row r="69" spans="3:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C69" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="D69" s="5"/>
-      <c r="E69" s="5"/>
-      <c r="F69" s="5"/>
-      <c r="G69" s="5"/>
-      <c r="H69" s="19" t="s">
-        <v>91</v>
-      </c>
-      <c r="I69" s="20"/>
-      <c r="J69" s="20"/>
-      <c r="K69" s="20"/>
-      <c r="L69" s="7"/>
+      <c r="C69" s="17" t="str">
+        <f>Project_Counteragent_Entity_Type&amp; " "&amp;Project_Counteragent_Name&amp;CHAR(10)&amp;CHAR(10)&amp;"(დამკვეთი)"&amp;CHAR(10)&amp;CHAR(10)&amp;CHAR(10)&amp;CHAR(10)&amp;"----------------------------------"&amp;CHAR(10)&amp;"დირექტორი" &amp;CHAR(10)&amp;Project_Counteragent_Director</f>
+        <v xml:space="preserve"> 
+(დამკვეთი)
+----------------------------------
+დირექტორი
+</v>
+      </c>
+      <c r="D69" s="18"/>
+      <c r="E69" s="18"/>
+      <c r="F69" s="18"/>
+      <c r="G69" s="18"/>
+      <c r="H69" s="17" t="str">
+        <f>Project_Insider_Entity_Type&amp; " "&amp;Project_Insider_Name&amp;CHAR(10)&amp;CHAR(10)&amp;"(შემსრულებელი)"&amp;CHAR(10)&amp;CHAR(10)&amp;CHAR(10)&amp;CHAR(10)&amp;"----------------------------------"&amp;CHAR(10)&amp;"დირექტორი" &amp;CHAR(10)&amp;Project_Insider_Director_Normative</f>
+        <v xml:space="preserve"> 
+(შემსრულებელი)
+----------------------------------
+დირექტორი
+</v>
+      </c>
+      <c r="I69" s="18"/>
+      <c r="J69" s="18"/>
+      <c r="K69" s="18"/>
+      <c r="L69" s="5"/>
     </row>
     <row r="70" spans="3:12" x14ac:dyDescent="0.25">
-      <c r="C70" s="5"/>
-      <c r="D70" s="5"/>
-      <c r="E70" s="5"/>
-      <c r="F70" s="5"/>
-      <c r="G70" s="5"/>
-      <c r="H70" s="20"/>
-      <c r="I70" s="20"/>
-      <c r="J70" s="20"/>
-      <c r="K70" s="20"/>
-      <c r="L70" s="7"/>
+      <c r="C70" s="18"/>
+      <c r="D70" s="18"/>
+      <c r="E70" s="18"/>
+      <c r="F70" s="18"/>
+      <c r="G70" s="18"/>
+      <c r="H70" s="18"/>
+      <c r="I70" s="18"/>
+      <c r="J70" s="18"/>
+      <c r="K70" s="18"/>
+      <c r="L70" s="5"/>
     </row>
     <row r="71" spans="3:12" x14ac:dyDescent="0.25">
-      <c r="C71" s="5"/>
-      <c r="D71" s="5"/>
-      <c r="E71" s="5"/>
-      <c r="F71" s="5"/>
-      <c r="G71" s="5"/>
-      <c r="H71" s="20"/>
-      <c r="I71" s="20"/>
-      <c r="J71" s="20"/>
-      <c r="K71" s="20"/>
-      <c r="L71" s="7"/>
+      <c r="C71" s="18"/>
+      <c r="D71" s="18"/>
+      <c r="E71" s="18"/>
+      <c r="F71" s="18"/>
+      <c r="G71" s="18"/>
+      <c r="H71" s="18"/>
+      <c r="I71" s="18"/>
+      <c r="J71" s="18"/>
+      <c r="K71" s="18"/>
+      <c r="L71" s="5"/>
     </row>
     <row r="72" spans="3:12" x14ac:dyDescent="0.25">
-      <c r="C72" s="5"/>
-      <c r="D72" s="5"/>
-      <c r="E72" s="5"/>
-      <c r="F72" s="5"/>
-      <c r="G72" s="5"/>
-      <c r="H72" s="20"/>
-      <c r="I72" s="20"/>
-      <c r="J72" s="20"/>
-      <c r="K72" s="20"/>
-      <c r="L72" s="7"/>
+      <c r="C72" s="18"/>
+      <c r="D72" s="18"/>
+      <c r="E72" s="18"/>
+      <c r="F72" s="18"/>
+      <c r="G72" s="18"/>
+      <c r="H72" s="18"/>
+      <c r="I72" s="18"/>
+      <c r="J72" s="18"/>
+      <c r="K72" s="18"/>
+      <c r="L72" s="5"/>
     </row>
     <row r="73" spans="3:12" x14ac:dyDescent="0.25">
-      <c r="C73" s="5"/>
-      <c r="D73" s="5"/>
-      <c r="E73" s="5"/>
-      <c r="F73" s="5"/>
-      <c r="G73" s="5"/>
-      <c r="H73" s="20"/>
-      <c r="I73" s="20"/>
-      <c r="J73" s="20"/>
-      <c r="K73" s="20"/>
-      <c r="L73" s="7"/>
+      <c r="C73" s="18"/>
+      <c r="D73" s="18"/>
+      <c r="E73" s="18"/>
+      <c r="F73" s="18"/>
+      <c r="G73" s="18"/>
+      <c r="H73" s="18"/>
+      <c r="I73" s="18"/>
+      <c r="J73" s="18"/>
+      <c r="K73" s="18"/>
+      <c r="L73" s="5"/>
     </row>
     <row r="74" spans="3:12" x14ac:dyDescent="0.25">
-      <c r="C74" s="5"/>
-      <c r="D74" s="5"/>
-      <c r="E74" s="5"/>
-      <c r="F74" s="5"/>
-      <c r="G74" s="5"/>
-      <c r="H74" s="20"/>
-      <c r="I74" s="20"/>
-      <c r="J74" s="20"/>
-      <c r="K74" s="20"/>
-      <c r="L74" s="7"/>
+      <c r="C74" s="18"/>
+      <c r="D74" s="18"/>
+      <c r="E74" s="18"/>
+      <c r="F74" s="18"/>
+      <c r="G74" s="18"/>
+      <c r="H74" s="18"/>
+      <c r="I74" s="18"/>
+      <c r="J74" s="18"/>
+      <c r="K74" s="18"/>
+      <c r="L74" s="5"/>
     </row>
     <row r="75" spans="3:12" x14ac:dyDescent="0.25">
-      <c r="C75" s="5"/>
-      <c r="D75" s="5"/>
-      <c r="E75" s="5"/>
-      <c r="F75" s="5"/>
-      <c r="G75" s="5"/>
-      <c r="H75" s="20"/>
-      <c r="I75" s="20"/>
-      <c r="J75" s="20"/>
-      <c r="K75" s="20"/>
-      <c r="L75" s="7"/>
+      <c r="C75" s="18"/>
+      <c r="D75" s="18"/>
+      <c r="E75" s="18"/>
+      <c r="F75" s="18"/>
+      <c r="G75" s="18"/>
+      <c r="H75" s="18"/>
+      <c r="I75" s="18"/>
+      <c r="J75" s="18"/>
+      <c r="K75" s="18"/>
+      <c r="L75" s="5"/>
     </row>
     <row r="76" spans="3:12" x14ac:dyDescent="0.25">
-      <c r="C76" s="5"/>
-      <c r="D76" s="5"/>
-      <c r="E76" s="5"/>
-      <c r="F76" s="5"/>
-      <c r="G76" s="5"/>
-      <c r="H76" s="20"/>
-      <c r="I76" s="20"/>
-      <c r="J76" s="20"/>
-      <c r="K76" s="20"/>
-      <c r="L76" s="7"/>
+      <c r="C76" s="18"/>
+      <c r="D76" s="18"/>
+      <c r="E76" s="18"/>
+      <c r="F76" s="18"/>
+      <c r="G76" s="18"/>
+      <c r="H76" s="18"/>
+      <c r="I76" s="18"/>
+      <c r="J76" s="18"/>
+      <c r="K76" s="18"/>
+      <c r="L76" s="5"/>
     </row>
     <row r="77" spans="3:12" x14ac:dyDescent="0.25">
-      <c r="C77" s="5"/>
-      <c r="D77" s="5"/>
-      <c r="E77" s="5"/>
-      <c r="F77" s="5"/>
-      <c r="G77" s="5"/>
-      <c r="H77" s="20"/>
-      <c r="I77" s="20"/>
-      <c r="J77" s="20"/>
-      <c r="K77" s="20"/>
-      <c r="L77" s="7"/>
+      <c r="C77" s="18"/>
+      <c r="D77" s="18"/>
+      <c r="E77" s="18"/>
+      <c r="F77" s="18"/>
+      <c r="G77" s="18"/>
+      <c r="H77" s="18"/>
+      <c r="I77" s="18"/>
+      <c r="J77" s="18"/>
+      <c r="K77" s="18"/>
+      <c r="L77" s="5"/>
     </row>
     <row r="78" spans="3:12" x14ac:dyDescent="0.25">
-      <c r="C78" s="5"/>
-      <c r="D78" s="5"/>
-      <c r="E78" s="5"/>
-      <c r="F78" s="5"/>
-      <c r="G78" s="5"/>
-      <c r="H78" s="20"/>
-      <c r="I78" s="20"/>
-      <c r="J78" s="20"/>
-      <c r="K78" s="20"/>
-      <c r="L78" s="7"/>
+      <c r="C78" s="18"/>
+      <c r="D78" s="18"/>
+      <c r="E78" s="18"/>
+      <c r="F78" s="18"/>
+      <c r="G78" s="18"/>
+      <c r="H78" s="18"/>
+      <c r="I78" s="18"/>
+      <c r="J78" s="18"/>
+      <c r="K78" s="18"/>
+      <c r="L78" s="5"/>
     </row>
     <row r="79" spans="3:12" x14ac:dyDescent="0.25">
-      <c r="C79" s="5"/>
-      <c r="D79" s="5"/>
-      <c r="E79" s="5"/>
-      <c r="F79" s="5"/>
-      <c r="G79" s="5"/>
-      <c r="H79" s="20"/>
-      <c r="I79" s="20"/>
-      <c r="J79" s="20"/>
-      <c r="K79" s="20"/>
-      <c r="L79" s="7"/>
+      <c r="C79" s="18"/>
+      <c r="D79" s="18"/>
+      <c r="E79" s="18"/>
+      <c r="F79" s="18"/>
+      <c r="G79" s="18"/>
+      <c r="H79" s="18"/>
+      <c r="I79" s="18"/>
+      <c r="J79" s="18"/>
+      <c r="K79" s="18"/>
+      <c r="L79" s="5"/>
     </row>
     <row r="80" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C80" s="4"/>
@@ -1929,9 +2085,8 @@
       <c r="D85" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="Q3:U3"/>
-    <mergeCell ref="V3:AC3"/>
+  <mergeCells count="10">
+    <mergeCell ref="P3:W3"/>
     <mergeCell ref="C6:K14"/>
     <mergeCell ref="C1:K1"/>
     <mergeCell ref="C66:K66"/>
@@ -1940,19 +2095,19 @@
     <mergeCell ref="C64:H64"/>
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="C4:E4"/>
-    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="I4:K4"/>
   </mergeCells>
   <printOptions headings="1" gridLines="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="1">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0675467D-43AF-4C81-932C-5A9EE6AB67C4}">
           <x14:formula1>
             <xm:f>Jobs!$M$2:$M$100</xm:f>
           </x14:formula1>
-          <xm:sqref>V3:AC3</xm:sqref>
+          <xm:sqref>P3:W3</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1961,9 +2116,134 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5B2909F-CBC3-41A4-B2F0-79C9D9F424AC}">
+  <sheetPr codeName="Sheet2"/>
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="36.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="76.125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" s="13"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="B5" s="15" t="str">
+        <f>IFERROR(LEFT(Project_Counteragent_Director,FIND(" ",Project_Counteragent_Director)-1)&amp;" "&amp;IF(RIGHT(TRIM(MID(Project_Counteragent_Director,FIND(" ",Project_Counteragent_Director)+1,LEN(Project_Counteragent_Director))),1)="ე",LEFT(TRIM(MID(Project_Counteragent_Director,FIND(" ",Project_Counteragent_Director)+1,LEN(Project_Counteragent_Director))),LEN(TRIM(MID(Project_Counteragent_Director,FIND(" ",Project_Counteragent_Director)+1,LEN(Project_Counteragent_Director))))-1)&amp;"ის",IF(RIGHT(TRIM(MID(Project_Counteragent_Director,FIND(" ",Project_Counteragent_Director)+1,LEN(Project_Counteragent_Director))),1)="ა",LEFT(TRIM(MID(Project_Counteragent_Director,FIND(" ",Project_Counteragent_Director)+1,LEN(Project_Counteragent_Director))),LEN(TRIM(MID(Project_Counteragent_Director,FIND(" ",Project_Counteragent_Director)+1,LEN(Project_Counteragent_Director))))-1)&amp;"ას",IF(RIGHT(TRIM(MID(Project_Counteragent_Director,FIND(" ",Project_Counteragent_Director)+1,LEN(Project_Counteragent_Director))),1)="ი",LEFT(TRIM(MID(Project_Counteragent_Director,FIND(" ",Project_Counteragent_Director)+1,LEN(Project_Counteragent_Director))),LEN(TRIM(MID(Project_Counteragent_Director,FIND(" ",Project_Counteragent_Director)+1,LEN(Project_Counteragent_Director))))-1)&amp;"ის",IF(RIGHT(TRIM(MID(Project_Counteragent_Director,FIND(" ",Project_Counteragent_Director)+1,LEN(Project_Counteragent_Director))),1)="ო",LEFT(TRIM(MID(Project_Counteragent_Director,FIND(" ",Project_Counteragent_Director)+1,LEN(Project_Counteragent_Director))),LEN(TRIM(MID(Project_Counteragent_Director,FIND(" ",Project_Counteragent_Director)+1,LEN(Project_Counteragent_Director))))-1)&amp;"ოს",TRIM(MID(Project_Counteragent_Director,FIND(" ",Project_Counteragent_Director)+1,LEN(Project_Counteragent_Director))))))),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>92</v>
+      </c>
+      <c r="E6" s="12"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B9" s="12"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="B16" s="15" t="str">
+        <f>IFERROR(LEFT(Project_Insider_Director_Normative,FIND(" ",Project_Insider_Director_Normative)-1)&amp;" "&amp;IF(RIGHT(TRIM(MID(Project_Insider_Director_Normative,FIND(" ",Project_Insider_Director_Normative)+1,LEN(Project_Insider_Director_Normative))),1)="ე",LEFT(TRIM(MID(Project_Insider_Director_Normative,FIND(" ",Project_Insider_Director_Normative)+1,LEN(Project_Insider_Director_Normative))),LEN(TRIM(MID(Project_Insider_Director_Normative,FIND(" ",Project_Insider_Director_Normative)+1,LEN(Project_Insider_Director_Normative))))-1)&amp;"ის",IF(RIGHT(TRIM(MID(Project_Insider_Director_Normative,FIND(" ",Project_Insider_Director_Normative)+1,LEN(Project_Insider_Director_Normative))),1)="ა",LEFT(TRIM(MID(Project_Insider_Director_Normative,FIND(" ",Project_Insider_Director_Normative)+1,LEN(Project_Insider_Director_Normative))),LEN(TRIM(MID(Project_Insider_Director_Normative,FIND(" ",Project_Insider_Director_Normative)+1,LEN(Project_Insider_Director_Normative))))-1)&amp;"ას",IF(RIGHT(TRIM(MID(Project_Insider_Director_Normative,FIND(" ",Project_Insider_Director_Normative)+1,LEN(Project_Insider_Director_Normative))),1)="ი",LEFT(TRIM(MID(Project_Insider_Director_Normative,FIND(" ",Project_Insider_Director_Normative)+1,LEN(Project_Insider_Director_Normative))),LEN(TRIM(MID(Project_Insider_Director_Normative,FIND(" ",Project_Insider_Director_Normative)+1,LEN(Project_Insider_Director_Normative))))-1)&amp;"ის",IF(RIGHT(TRIM(MID(Project_Insider_Director_Normative,FIND(" ",Project_Insider_Director_Normative)+1,LEN(Project_Insider_Director_Normative))),1)="ო",LEFT(TRIM(MID(Project_Insider_Director_Normative,FIND(" ",Project_Insider_Director_Normative)+1,LEN(Project_Insider_Director_Normative))),LEN(TRIM(MID(Project_Insider_Director_Normative,FIND(" ",Project_Insider_Director_Normative)+1,LEN(Project_Insider_Director_Normative))))-1)&amp;"ოს",TRIM(MID(Project_Insider_Director_Normative,FIND(" ",Project_Insider_Director_Normative)+1,LEN(Project_Insider_Director_Normative))))))),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="B18" s="15"/>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>103</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:N6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.75" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.5" bestFit="1" customWidth="1"/>
@@ -1981,64 +2261,64 @@
     <col min="14" max="14" width="13.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="F1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="G1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="14" t="s">
+      <c r="H1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="14" t="s">
+      <c r="I1" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="14" t="s">
+      <c r="J1" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="14" t="s">
+      <c r="K1" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="14" t="s">
+      <c r="L1" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="14" t="s">
+      <c r="M1" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="14" t="s">
+      <c r="N1" s="9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="14">
+      <c r="D2" s="9">
         <v>13</v>
       </c>
-      <c r="E2" s="14">
+      <c r="E2" s="9">
         <v>1000</v>
       </c>
       <c r="F2" s="1">
@@ -2059,30 +2339,30 @@
       <c r="K2" s="1">
         <v>118268.1</v>
       </c>
-      <c r="L2" s="14" t="s">
+      <c r="L2" s="9" t="s">
         <v>17</v>
       </c>
       <c r="M2" s="2">
         <v>46169</v>
       </c>
-      <c r="N2" s="14" t="s">
+      <c r="N2" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="14">
+      <c r="D3" s="9">
         <v>13</v>
       </c>
-      <c r="E3" s="14">
+      <c r="E3" s="9">
         <v>1600</v>
       </c>
       <c r="F3" s="1">
@@ -2103,30 +2383,30 @@
       <c r="K3" s="1">
         <v>147664.18</v>
       </c>
-      <c r="L3" s="14" t="s">
+      <c r="L3" s="9" t="s">
         <v>17</v>
       </c>
       <c r="M3" s="2">
         <v>46169</v>
       </c>
-      <c r="N3" s="14" t="s">
+      <c r="N3" s="9" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="14">
+      <c r="D4" s="9">
         <v>4</v>
       </c>
-      <c r="E4" s="14">
+      <c r="E4" s="9">
         <v>1000</v>
       </c>
       <c r="F4" s="1">
@@ -2147,30 +2427,30 @@
       <c r="K4" s="1">
         <v>0</v>
       </c>
-      <c r="L4" s="14" t="s">
+      <c r="L4" s="9" t="s">
         <v>17</v>
       </c>
       <c r="M4" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N4" s="14" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="14" t="s">
+      <c r="N4" s="9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C5" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="14">
+      <c r="D5" s="9">
         <v>4</v>
       </c>
-      <c r="E5" s="14">
+      <c r="E5" s="9">
         <v>1000</v>
       </c>
       <c r="F5" s="1">
@@ -2191,30 +2471,30 @@
       <c r="K5" s="1">
         <v>0</v>
       </c>
-      <c r="L5" s="14" t="s">
+      <c r="L5" s="9" t="s">
         <v>17</v>
       </c>
       <c r="M5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N5" s="14" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="E6" s="14" t="s">
+      <c r="N5" s="9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="9" t="s">
         <v>24</v>
       </c>
       <c r="F6" s="1">
@@ -2235,13 +2515,13 @@
       <c r="K6" s="1">
         <v>265932.28000000003</v>
       </c>
-      <c r="L6" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="M6" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="N6" s="14" t="s">
+      <c r="L6" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="M6" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="N6" s="9" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2250,10 +2530,11 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.125" bestFit="1" customWidth="1"/>
@@ -2263,7 +2544,7 @@
     <col min="8" max="8" width="8.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>27</v>
       </c>
@@ -2289,7 +2570,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>45561</v>
       </c>
@@ -2315,7 +2596,7 @@
         <v>10.85</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>45567</v>
       </c>
@@ -2341,7 +2622,7 @@
         <v>10334.9</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>45463</v>
       </c>
@@ -2367,7 +2648,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>24</v>
       </c>
@@ -2393,7 +2674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>24</v>
       </c>
@@ -2419,7 +2700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>45394</v>
       </c>
@@ -2453,10 +2734,11 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:P24"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.5" bestFit="1" customWidth="1"/>
@@ -2476,7 +2758,7 @@
     <col min="16" max="16" width="29.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>47</v>
       </c>
@@ -2526,7 +2808,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>45561</v>
       </c>
@@ -2576,7 +2858,7 @@
         <v>22310.713914</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>45561</v>
       </c>
@@ -2626,7 +2908,7 @@
         <v>18004.996085999996</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>45466</v>
       </c>
@@ -2676,7 +2958,7 @@
         <v>208.18465</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>45466</v>
       </c>
@@ -2726,7 +3008,7 @@
         <v>20714.372674999999</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>45466</v>
       </c>
@@ -2776,7 +3058,7 @@
         <v>20714.372674999999</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>45463</v>
       </c>
@@ -2826,7 +3108,7 @@
         <v>4005.5674279999994</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>45463</v>
       </c>
@@ -2876,7 +3158,7 @@
         <v>3913.8139119999996</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>45463</v>
       </c>
@@ -2926,7 +3208,7 @@
         <v>3913.8139119999996</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>45463</v>
       </c>
@@ -2976,7 +3258,7 @@
         <v>3208.3647479999995</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>45463</v>
       </c>
@@ -3026,7 +3308,7 @@
         <v>1880.2</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>45463</v>
       </c>
@@ -3076,7 +3358,7 @@
         <v>1880.2</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>45394</v>
       </c>
@@ -3126,7 +3408,7 @@
         <v>53757.627035999998</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>45394</v>
       </c>
@@ -3176,7 +3458,7 @@
         <v>44068.031693999998</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>45394</v>
       </c>
@@ -3226,7 +3508,7 @@
         <v>55017.894233999992</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>45394</v>
       </c>
@@ -3276,7 +3558,7 @@
         <v>53757.627035999998</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>45394</v>
       </c>
@@ -3326,7 +3608,7 @@
         <v>1862.7249639999998</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>45394</v>
       </c>
@@ -3376,7 +3658,7 @@
         <v>1526.9763059999998</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>45394</v>
       </c>
@@ -3426,7 +3708,7 @@
         <v>1906.3937659999997</v>
       </c>
     </row>
-    <row r="20" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>45394</v>
       </c>
@@ -3476,7 +3758,7 @@
         <v>1862.7249639999998</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>45327</v>
       </c>
@@ -3526,7 +3808,7 @@
         <v>56856.115199999993</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>45327</v>
       </c>
@@ -3576,7 +3858,7 @@
         <v>45540.403200000001</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>45327</v>
       </c>
@@ -3626,7 +3908,7 @@
         <v>55553.7408</v>
       </c>
     </row>
-    <row r="24" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>45327</v>
       </c>

</xml_diff>